<commit_message>
create option for inventory
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Laravel\software_access_managements\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\backend\financial_project\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -137,7 +137,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -192,6 +192,11 @@
       <sz val="16"/>
       <color theme="1"/>
       <name val="Khmer OS Muol Light"/>
+    </font>
+    <font>
+      <sz val="26"/>
+      <color theme="1"/>
+      <name val="Tacteing"/>
     </font>
   </fonts>
   <fills count="2">
@@ -338,39 +343,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -384,17 +356,50 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -736,7 +741,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:X100"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="25.5"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="25.5" x14ac:dyDescent="0.7"/>
   <cols>
     <col min="1" max="1" width="7.875" style="20" customWidth="1"/>
     <col min="2" max="2" width="9.375" style="20" customWidth="1"/>
@@ -752,86 +757,86 @@
     <col min="16" max="16" width="19.375" style="17" customWidth="1"/>
     <col min="17" max="17" width="18.375" style="17" customWidth="1"/>
     <col min="18" max="18" width="15.625" style="18" customWidth="1"/>
-    <col min="19" max="19" width="13" style="45" customWidth="1"/>
+    <col min="19" max="19" width="13" style="33" customWidth="1"/>
     <col min="20" max="20" width="13" style="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="33">
-      <c r="A1" s="32" t="s">
+    <row r="1" spans="1:24" ht="33" x14ac:dyDescent="0.25">
+      <c r="A1" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="32"/>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="32"/>
-      <c r="R1" s="32"/>
-      <c r="S1" s="32"/>
-      <c r="T1" s="32"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
       <c r="U1" s="2"/>
     </row>
-    <row r="2" spans="1:24">
-      <c r="A2" s="33" t="s">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A2" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
-      <c r="J2" s="33"/>
-      <c r="K2" s="33"/>
-      <c r="L2" s="33"/>
-      <c r="M2" s="33"/>
-      <c r="N2" s="33"/>
-      <c r="O2" s="33"/>
-      <c r="P2" s="33"/>
-      <c r="Q2" s="33"/>
-      <c r="R2" s="33"/>
-      <c r="S2" s="33"/>
-      <c r="T2" s="33"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
+      <c r="N2" s="36"/>
+      <c r="O2" s="36"/>
+      <c r="P2" s="36"/>
+      <c r="Q2" s="36"/>
+      <c r="R2" s="36"/>
+      <c r="S2" s="36"/>
+      <c r="T2" s="36"/>
       <c r="U2" s="4"/>
     </row>
-    <row r="3" spans="1:24" ht="33">
-      <c r="A3" s="34">
+    <row r="3" spans="1:24" ht="29.25" x14ac:dyDescent="0.25">
+      <c r="A3" s="45">
         <v>3</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
-      <c r="K3" s="34"/>
-      <c r="L3" s="34"/>
-      <c r="M3" s="34"/>
-      <c r="N3" s="34"/>
-      <c r="O3" s="34"/>
-      <c r="P3" s="34"/>
-      <c r="Q3" s="34"/>
-      <c r="R3" s="34"/>
-      <c r="S3" s="34"/>
-      <c r="T3" s="34"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="45"/>
+      <c r="J3" s="45"/>
+      <c r="K3" s="45"/>
+      <c r="L3" s="45"/>
+      <c r="M3" s="45"/>
+      <c r="N3" s="45"/>
+      <c r="O3" s="45"/>
+      <c r="P3" s="45"/>
+      <c r="Q3" s="45"/>
+      <c r="R3" s="45"/>
+      <c r="S3" s="45"/>
+      <c r="T3" s="45"/>
       <c r="U3" s="5"/>
     </row>
-    <row r="4" spans="1:24" ht="33">
+    <row r="4" spans="1:24" ht="33" x14ac:dyDescent="0.7">
       <c r="A4" s="25" t="s">
         <v>0</v>
       </c>
@@ -856,7 +861,7 @@
       <c r="T4" s="11"/>
       <c r="U4" s="1"/>
     </row>
-    <row r="5" spans="1:24" ht="33">
+    <row r="5" spans="1:24" ht="33" x14ac:dyDescent="0.7">
       <c r="A5" s="25" t="s">
         <v>1</v>
       </c>
@@ -881,7 +886,7 @@
       <c r="T5" s="11"/>
       <c r="U5" s="1"/>
     </row>
-    <row r="6" spans="1:24" ht="33">
+    <row r="6" spans="1:24" ht="33" x14ac:dyDescent="0.7">
       <c r="A6" s="25" t="s">
         <v>2</v>
       </c>
@@ -906,7 +911,7 @@
       <c r="T6" s="12"/>
       <c r="U6" s="1"/>
     </row>
-    <row r="7" spans="1:24" ht="33">
+    <row r="7" spans="1:24" ht="33" x14ac:dyDescent="0.7">
       <c r="A7" s="25" t="s">
         <v>3</v>
       </c>
@@ -931,7 +936,7 @@
       <c r="T7" s="12"/>
       <c r="U7" s="1"/>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.7">
       <c r="A8" s="13"/>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -954,152 +959,152 @@
       <c r="T8" s="16"/>
       <c r="U8" s="1"/>
     </row>
-    <row r="9" spans="1:24" ht="29.25">
-      <c r="A9" s="35" t="s">
+    <row r="9" spans="1:24" ht="29.25" x14ac:dyDescent="0.25">
+      <c r="A9" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="35"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
-      <c r="J9" s="35"/>
-      <c r="K9" s="35"/>
-      <c r="L9" s="35"/>
-      <c r="M9" s="35"/>
-      <c r="N9" s="35"/>
-      <c r="O9" s="35"/>
-      <c r="P9" s="35"/>
-      <c r="Q9" s="35"/>
-      <c r="R9" s="35"/>
-      <c r="S9" s="35"/>
-      <c r="T9" s="35"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="37"/>
+      <c r="K9" s="37"/>
+      <c r="L9" s="37"/>
+      <c r="M9" s="37"/>
+      <c r="N9" s="37"/>
+      <c r="O9" s="37"/>
+      <c r="P9" s="37"/>
+      <c r="Q9" s="37"/>
+      <c r="R9" s="37"/>
+      <c r="S9" s="37"/>
+      <c r="T9" s="37"/>
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
       <c r="W9" s="2"/>
       <c r="X9" s="2"/>
     </row>
-    <row r="10" spans="1:24">
-      <c r="A10" s="36" t="s">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.7">
+      <c r="A10" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="36"/>
-      <c r="C10" s="36"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="36"/>
-      <c r="G10" s="36"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="36"/>
-      <c r="J10" s="36"/>
-      <c r="K10" s="36"/>
-      <c r="L10" s="36"/>
-      <c r="M10" s="36"/>
-      <c r="N10" s="36"/>
-      <c r="O10" s="36"/>
-      <c r="P10" s="36"/>
-      <c r="Q10" s="36"/>
-      <c r="R10" s="36"/>
-      <c r="S10" s="36"/>
-      <c r="T10" s="36"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="34"/>
+      <c r="J10" s="34"/>
+      <c r="K10" s="34"/>
+      <c r="L10" s="34"/>
+      <c r="M10" s="34"/>
+      <c r="N10" s="34"/>
+      <c r="O10" s="34"/>
+      <c r="P10" s="34"/>
+      <c r="Q10" s="34"/>
+      <c r="R10" s="34"/>
+      <c r="S10" s="34"/>
+      <c r="T10" s="34"/>
       <c r="U10" s="3"/>
       <c r="V10" s="3"/>
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
     </row>
-    <row r="11" spans="1:24">
-      <c r="A11" s="28" t="s">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A11" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="28" t="s">
+      <c r="B11" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="28" t="s">
+      <c r="D11" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="28" t="s">
+      <c r="E11" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="29" t="s">
+      <c r="F11" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="29" t="s">
+      <c r="G11" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="H11" s="30" t="s">
+      <c r="H11" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="I11" s="30"/>
-      <c r="J11" s="30"/>
-      <c r="K11" s="30"/>
-      <c r="L11" s="30"/>
-      <c r="M11" s="31" t="s">
+      <c r="I11" s="39"/>
+      <c r="J11" s="39"/>
+      <c r="K11" s="39"/>
+      <c r="L11" s="39"/>
+      <c r="M11" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="N11" s="30" t="s">
+      <c r="N11" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="O11" s="30" t="s">
+      <c r="O11" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="P11" s="30" t="s">
+      <c r="P11" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="Q11" s="30" t="s">
+      <c r="Q11" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="R11" s="31" t="s">
+      <c r="R11" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="S11" s="26" t="s">
+      <c r="S11" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="T11" s="26"/>
-    </row>
-    <row r="12" spans="1:24">
-      <c r="A12" s="28"/>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="29"/>
-      <c r="G12" s="29"/>
-      <c r="H12" s="30" t="s">
+      <c r="T11" s="40"/>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A12" s="38"/>
+      <c r="B12" s="38"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="I12" s="30"/>
-      <c r="J12" s="30"/>
-      <c r="K12" s="30"/>
-      <c r="L12" s="30" t="s">
+      <c r="I12" s="39"/>
+      <c r="J12" s="39"/>
+      <c r="K12" s="39"/>
+      <c r="L12" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="M12" s="31"/>
-      <c r="N12" s="30"/>
-      <c r="O12" s="30"/>
-      <c r="P12" s="30"/>
-      <c r="Q12" s="30"/>
-      <c r="R12" s="31"/>
-      <c r="S12" s="42" t="s">
+      <c r="M12" s="44"/>
+      <c r="N12" s="39"/>
+      <c r="O12" s="39"/>
+      <c r="P12" s="39"/>
+      <c r="Q12" s="39"/>
+      <c r="R12" s="44"/>
+      <c r="S12" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="T12" s="27" t="s">
+      <c r="T12" s="42" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:24" ht="51">
-      <c r="A13" s="28"/>
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="29"/>
-      <c r="G13" s="29"/>
+    <row r="13" spans="1:24" ht="51" x14ac:dyDescent="0.25">
+      <c r="A13" s="38"/>
+      <c r="B13" s="38"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="43"/>
+      <c r="G13" s="43"/>
       <c r="H13" s="23" t="s">
         <v>28</v>
       </c>
@@ -1112,323 +1117,311 @@
       <c r="K13" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="L13" s="30"/>
-      <c r="M13" s="31"/>
-      <c r="N13" s="30"/>
-      <c r="O13" s="30"/>
-      <c r="P13" s="30"/>
-      <c r="Q13" s="30"/>
-      <c r="R13" s="31"/>
-      <c r="S13" s="42"/>
-      <c r="T13" s="27"/>
-    </row>
-    <row r="14" spans="1:24">
-      <c r="A14" s="37"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="40"/>
-      <c r="G14" s="40"/>
-      <c r="H14" s="40"/>
-      <c r="I14" s="40"/>
-      <c r="J14" s="40"/>
-      <c r="K14" s="40"/>
-      <c r="L14" s="40"/>
-      <c r="M14" s="41"/>
-      <c r="N14" s="40"/>
-      <c r="O14" s="40"/>
-      <c r="P14" s="40"/>
-      <c r="Q14" s="40"/>
-      <c r="R14" s="41"/>
-      <c r="S14" s="43"/>
+      <c r="L13" s="39"/>
+      <c r="M13" s="44"/>
+      <c r="N13" s="39"/>
+      <c r="O13" s="39"/>
+      <c r="P13" s="39"/>
+      <c r="Q13" s="39"/>
+      <c r="R13" s="44"/>
+      <c r="S13" s="41"/>
+      <c r="T13" s="42"/>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.7">
+      <c r="A14" s="26"/>
+      <c r="B14" s="26"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="29"/>
+      <c r="K14" s="29"/>
+      <c r="L14" s="29"/>
+      <c r="M14" s="30"/>
+      <c r="N14" s="29"/>
+      <c r="O14" s="29"/>
+      <c r="P14" s="29"/>
+      <c r="Q14" s="29"/>
+      <c r="R14" s="30"/>
+      <c r="S14" s="31"/>
       <c r="T14" s="24"/>
       <c r="U14" s="1"/>
     </row>
-    <row r="15" spans="1:24">
-      <c r="S15" s="44"/>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.7">
+      <c r="S15" s="32"/>
       <c r="T15" s="24"/>
       <c r="U15" s="1"/>
     </row>
-    <row r="16" spans="1:24">
-      <c r="S16" s="44"/>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.7">
+      <c r="S16" s="32"/>
       <c r="T16" s="24"/>
       <c r="U16" s="1"/>
     </row>
-    <row r="17" spans="19:21">
-      <c r="S17" s="44"/>
+    <row r="17" spans="19:21" x14ac:dyDescent="0.7">
+      <c r="S17" s="32"/>
       <c r="T17" s="24"/>
       <c r="U17" s="1"/>
     </row>
-    <row r="18" spans="19:21">
-      <c r="S18" s="44"/>
+    <row r="18" spans="19:21" x14ac:dyDescent="0.7">
+      <c r="S18" s="32"/>
       <c r="T18" s="24"/>
       <c r="U18" s="1"/>
     </row>
-    <row r="19" spans="19:21">
-      <c r="S19" s="44"/>
+    <row r="19" spans="19:21" x14ac:dyDescent="0.7">
+      <c r="S19" s="32"/>
       <c r="T19" s="24"/>
       <c r="U19" s="1"/>
     </row>
-    <row r="20" spans="19:21">
-      <c r="S20" s="44"/>
+    <row r="20" spans="19:21" x14ac:dyDescent="0.7">
+      <c r="S20" s="32"/>
       <c r="T20" s="24"/>
       <c r="U20" s="1"/>
     </row>
-    <row r="21" spans="19:21">
+    <row r="21" spans="19:21" x14ac:dyDescent="0.7">
       <c r="U21" s="1"/>
     </row>
-    <row r="22" spans="19:21">
+    <row r="22" spans="19:21" x14ac:dyDescent="0.7">
       <c r="U22" s="1"/>
     </row>
-    <row r="23" spans="19:21">
+    <row r="23" spans="19:21" x14ac:dyDescent="0.7">
       <c r="U23" s="1"/>
     </row>
-    <row r="24" spans="19:21">
+    <row r="24" spans="19:21" x14ac:dyDescent="0.7">
       <c r="U24" s="1"/>
     </row>
-    <row r="25" spans="19:21">
+    <row r="25" spans="19:21" x14ac:dyDescent="0.7">
       <c r="U25" s="1"/>
     </row>
-    <row r="26" spans="19:21">
+    <row r="26" spans="19:21" x14ac:dyDescent="0.7">
       <c r="U26" s="1"/>
     </row>
-    <row r="27" spans="19:21">
+    <row r="27" spans="19:21" x14ac:dyDescent="0.7">
       <c r="U27" s="1"/>
     </row>
-    <row r="28" spans="19:21">
+    <row r="28" spans="19:21" x14ac:dyDescent="0.7">
       <c r="U28" s="1"/>
     </row>
-    <row r="29" spans="19:21">
+    <row r="29" spans="19:21" x14ac:dyDescent="0.7">
       <c r="U29" s="1"/>
     </row>
-    <row r="30" spans="19:21">
+    <row r="30" spans="19:21" x14ac:dyDescent="0.7">
       <c r="U30" s="1"/>
     </row>
-    <row r="31" spans="19:21">
+    <row r="31" spans="19:21" x14ac:dyDescent="0.7">
       <c r="U31" s="1"/>
     </row>
-    <row r="32" spans="19:21">
+    <row r="32" spans="19:21" x14ac:dyDescent="0.7">
       <c r="U32" s="1"/>
     </row>
-    <row r="33" spans="21:21">
+    <row r="33" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U33" s="1"/>
     </row>
-    <row r="34" spans="21:21">
+    <row r="34" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U34" s="1"/>
     </row>
-    <row r="35" spans="21:21">
+    <row r="35" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U35" s="1"/>
     </row>
-    <row r="36" spans="21:21">
+    <row r="36" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U36" s="1"/>
     </row>
-    <row r="37" spans="21:21">
+    <row r="37" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U37" s="1"/>
     </row>
-    <row r="38" spans="21:21">
+    <row r="38" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U38" s="1"/>
     </row>
-    <row r="39" spans="21:21">
+    <row r="39" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U39" s="1"/>
     </row>
-    <row r="40" spans="21:21">
+    <row r="40" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U40" s="1"/>
     </row>
-    <row r="41" spans="21:21">
+    <row r="41" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U41" s="1"/>
     </row>
-    <row r="42" spans="21:21">
+    <row r="42" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U42" s="1"/>
     </row>
-    <row r="43" spans="21:21">
+    <row r="43" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U43" s="1"/>
     </row>
-    <row r="44" spans="21:21">
+    <row r="44" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U44" s="1"/>
     </row>
-    <row r="45" spans="21:21">
+    <row r="45" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U45" s="1"/>
     </row>
-    <row r="46" spans="21:21">
+    <row r="46" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U46" s="1"/>
     </row>
-    <row r="47" spans="21:21">
+    <row r="47" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U47" s="1"/>
     </row>
-    <row r="48" spans="21:21">
+    <row r="48" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U48" s="1"/>
     </row>
-    <row r="49" spans="21:21">
+    <row r="49" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U49" s="1"/>
     </row>
-    <row r="50" spans="21:21">
+    <row r="50" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U50" s="1"/>
     </row>
-    <row r="51" spans="21:21">
+    <row r="51" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U51" s="1"/>
     </row>
-    <row r="52" spans="21:21">
+    <row r="52" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U52" s="1"/>
     </row>
-    <row r="53" spans="21:21">
+    <row r="53" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U53" s="1"/>
     </row>
-    <row r="54" spans="21:21">
+    <row r="54" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U54" s="1"/>
     </row>
-    <row r="55" spans="21:21">
+    <row r="55" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U55" s="1"/>
     </row>
-    <row r="56" spans="21:21">
+    <row r="56" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U56" s="1"/>
     </row>
-    <row r="57" spans="21:21">
+    <row r="57" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U57" s="1"/>
     </row>
-    <row r="58" spans="21:21">
+    <row r="58" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U58" s="1"/>
     </row>
-    <row r="59" spans="21:21">
+    <row r="59" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U59" s="1"/>
     </row>
-    <row r="60" spans="21:21">
+    <row r="60" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U60" s="1"/>
     </row>
-    <row r="61" spans="21:21">
+    <row r="61" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U61" s="1"/>
     </row>
-    <row r="62" spans="21:21">
+    <row r="62" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U62" s="1"/>
     </row>
-    <row r="63" spans="21:21">
+    <row r="63" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U63" s="1"/>
     </row>
-    <row r="64" spans="21:21">
+    <row r="64" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U64" s="1"/>
     </row>
-    <row r="65" spans="21:21">
+    <row r="65" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U65" s="1"/>
     </row>
-    <row r="66" spans="21:21">
+    <row r="66" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U66" s="1"/>
     </row>
-    <row r="67" spans="21:21">
+    <row r="67" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U67" s="1"/>
     </row>
-    <row r="68" spans="21:21">
+    <row r="68" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U68" s="1"/>
     </row>
-    <row r="69" spans="21:21">
+    <row r="69" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U69" s="1"/>
     </row>
-    <row r="70" spans="21:21">
+    <row r="70" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U70" s="1"/>
     </row>
-    <row r="71" spans="21:21">
+    <row r="71" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U71" s="1"/>
     </row>
-    <row r="72" spans="21:21">
+    <row r="72" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U72" s="1"/>
     </row>
-    <row r="73" spans="21:21">
+    <row r="73" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U73" s="1"/>
     </row>
-    <row r="74" spans="21:21">
+    <row r="74" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U74" s="1"/>
     </row>
-    <row r="75" spans="21:21">
+    <row r="75" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U75" s="1"/>
     </row>
-    <row r="76" spans="21:21">
+    <row r="76" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U76" s="1"/>
     </row>
-    <row r="77" spans="21:21">
+    <row r="77" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U77" s="1"/>
     </row>
-    <row r="78" spans="21:21">
+    <row r="78" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U78" s="1"/>
     </row>
-    <row r="79" spans="21:21">
+    <row r="79" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U79" s="1"/>
     </row>
-    <row r="80" spans="21:21">
+    <row r="80" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U80" s="1"/>
     </row>
-    <row r="81" spans="21:21">
+    <row r="81" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U81" s="1"/>
     </row>
-    <row r="82" spans="21:21">
+    <row r="82" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U82" s="1"/>
     </row>
-    <row r="83" spans="21:21">
+    <row r="83" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U83" s="1"/>
     </row>
-    <row r="84" spans="21:21">
+    <row r="84" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U84" s="1"/>
     </row>
-    <row r="85" spans="21:21">
+    <row r="85" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U85" s="1"/>
     </row>
-    <row r="86" spans="21:21">
+    <row r="86" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U86" s="1"/>
     </row>
-    <row r="87" spans="21:21">
+    <row r="87" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U87" s="1"/>
     </row>
-    <row r="88" spans="21:21">
+    <row r="88" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U88" s="1"/>
     </row>
-    <row r="89" spans="21:21">
+    <row r="89" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U89" s="1"/>
     </row>
-    <row r="90" spans="21:21">
+    <row r="90" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U90" s="1"/>
     </row>
-    <row r="91" spans="21:21">
+    <row r="91" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U91" s="1"/>
     </row>
-    <row r="92" spans="21:21">
+    <row r="92" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U92" s="1"/>
     </row>
-    <row r="93" spans="21:21">
+    <row r="93" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U93" s="1"/>
     </row>
-    <row r="94" spans="21:21">
+    <row r="94" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U94" s="1"/>
     </row>
-    <row r="95" spans="21:21">
+    <row r="95" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U95" s="1"/>
     </row>
-    <row r="96" spans="21:21">
+    <row r="96" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U96" s="1"/>
     </row>
-    <row r="97" spans="21:21">
+    <row r="97" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U97" s="1"/>
     </row>
-    <row r="98" spans="21:21">
+    <row r="98" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U98" s="1"/>
     </row>
-    <row r="99" spans="21:21">
+    <row r="99" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U99" s="1"/>
     </row>
-    <row r="100" spans="21:21">
+    <row r="100" spans="21:21" x14ac:dyDescent="0.7">
       <c r="U100" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A10:T10"/>
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="A2:T2"/>
-    <mergeCell ref="A3:T3"/>
-    <mergeCell ref="A9:T9"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="D11:D13"/>
-    <mergeCell ref="H11:L11"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="L12:L13"/>
     <mergeCell ref="S11:T11"/>
     <mergeCell ref="S12:S13"/>
     <mergeCell ref="T12:T13"/>
@@ -1441,6 +1434,18 @@
     <mergeCell ref="N11:N13"/>
     <mergeCell ref="O11:O13"/>
     <mergeCell ref="M11:M13"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="D11:D13"/>
+    <mergeCell ref="H11:L11"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="L12:L13"/>
+    <mergeCell ref="A10:T10"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A2:T2"/>
+    <mergeCell ref="A3:T3"/>
+    <mergeCell ref="A9:T9"/>
   </mergeCells>
   <conditionalFormatting sqref="T4:T8 T11:T1048576">
     <cfRule type="cellIs" dxfId="3" priority="4" operator="lessThan">

</xml_diff>

<commit_message>
add export methods for download
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -365,6 +365,27 @@
     <xf numFmtId="10" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -374,32 +395,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -762,78 +762,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="33" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
-      <c r="S1" s="35"/>
-      <c r="T1" s="35"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="42"/>
+      <c r="R1" s="42"/>
+      <c r="S1" s="42"/>
+      <c r="T1" s="42"/>
       <c r="U1" s="2"/>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
-      <c r="P2" s="36"/>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
-      <c r="T2" s="36"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
+      <c r="P2" s="43"/>
+      <c r="Q2" s="43"/>
+      <c r="R2" s="43"/>
+      <c r="S2" s="43"/>
+      <c r="T2" s="43"/>
       <c r="U2" s="4"/>
     </row>
     <row r="3" spans="1:24" ht="29.25" x14ac:dyDescent="0.25">
-      <c r="A3" s="45">
+      <c r="A3" s="44">
         <v>3</v>
       </c>
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="45"/>
-      <c r="I3" s="45"/>
-      <c r="J3" s="45"/>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
-      <c r="M3" s="45"/>
-      <c r="N3" s="45"/>
-      <c r="O3" s="45"/>
-      <c r="P3" s="45"/>
-      <c r="Q3" s="45"/>
-      <c r="R3" s="45"/>
-      <c r="S3" s="45"/>
-      <c r="T3" s="45"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="44"/>
+      <c r="O3" s="44"/>
+      <c r="P3" s="44"/>
+      <c r="Q3" s="44"/>
+      <c r="R3" s="44"/>
+      <c r="S3" s="44"/>
+      <c r="T3" s="44"/>
       <c r="U3" s="5"/>
     </row>
     <row r="4" spans="1:24" ht="33" x14ac:dyDescent="0.7">
@@ -960,81 +960,81 @@
       <c r="U8" s="1"/>
     </row>
     <row r="9" spans="1:24" ht="29.25" x14ac:dyDescent="0.25">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="37"/>
-      <c r="K9" s="37"/>
-      <c r="L9" s="37"/>
-      <c r="M9" s="37"/>
-      <c r="N9" s="37"/>
-      <c r="O9" s="37"/>
-      <c r="P9" s="37"/>
-      <c r="Q9" s="37"/>
-      <c r="R9" s="37"/>
-      <c r="S9" s="37"/>
-      <c r="T9" s="37"/>
+      <c r="B9" s="45"/>
+      <c r="C9" s="45"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45"/>
+      <c r="G9" s="45"/>
+      <c r="H9" s="45"/>
+      <c r="I9" s="45"/>
+      <c r="J9" s="45"/>
+      <c r="K9" s="45"/>
+      <c r="L9" s="45"/>
+      <c r="M9" s="45"/>
+      <c r="N9" s="45"/>
+      <c r="O9" s="45"/>
+      <c r="P9" s="45"/>
+      <c r="Q9" s="45"/>
+      <c r="R9" s="45"/>
+      <c r="S9" s="45"/>
+      <c r="T9" s="45"/>
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
       <c r="W9" s="2"/>
       <c r="X9" s="2"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.7">
-      <c r="A10" s="34" t="s">
+      <c r="A10" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="34"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="34"/>
-      <c r="I10" s="34"/>
-      <c r="J10" s="34"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="34"/>
-      <c r="M10" s="34"/>
-      <c r="N10" s="34"/>
-      <c r="O10" s="34"/>
-      <c r="P10" s="34"/>
-      <c r="Q10" s="34"/>
-      <c r="R10" s="34"/>
-      <c r="S10" s="34"/>
-      <c r="T10" s="34"/>
+      <c r="B10" s="41"/>
+      <c r="C10" s="41"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="41"/>
+      <c r="H10" s="41"/>
+      <c r="I10" s="41"/>
+      <c r="J10" s="41"/>
+      <c r="K10" s="41"/>
+      <c r="L10" s="41"/>
+      <c r="M10" s="41"/>
+      <c r="N10" s="41"/>
+      <c r="O10" s="41"/>
+      <c r="P10" s="41"/>
+      <c r="Q10" s="41"/>
+      <c r="R10" s="41"/>
+      <c r="S10" s="41"/>
+      <c r="T10" s="41"/>
       <c r="U10" s="3"/>
       <c r="V10" s="3"/>
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A11" s="38" t="s">
+      <c r="A11" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="38" t="s">
+      <c r="B11" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="38" t="s">
+      <c r="C11" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="38" t="s">
+      <c r="E11" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="43" t="s">
+      <c r="F11" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="43" t="s">
+      <c r="G11" s="38" t="s">
         <v>14</v>
       </c>
       <c r="H11" s="39" t="s">
@@ -1044,7 +1044,7 @@
       <c r="J11" s="39"/>
       <c r="K11" s="39"/>
       <c r="L11" s="39"/>
-      <c r="M11" s="44" t="s">
+      <c r="M11" s="40" t="s">
         <v>30</v>
       </c>
       <c r="N11" s="39" t="s">
@@ -1059,22 +1059,22 @@
       <c r="Q11" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="R11" s="44" t="s">
+      <c r="R11" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="S11" s="40" t="s">
+      <c r="S11" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="T11" s="40"/>
+      <c r="T11" s="34"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" s="38"/>
-      <c r="B12" s="38"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
+      <c r="A12" s="37"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="38"/>
       <c r="H12" s="39" t="s">
         <v>22</v>
       </c>
@@ -1084,27 +1084,27 @@
       <c r="L12" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="M12" s="44"/>
+      <c r="M12" s="40"/>
       <c r="N12" s="39"/>
       <c r="O12" s="39"/>
       <c r="P12" s="39"/>
       <c r="Q12" s="39"/>
-      <c r="R12" s="44"/>
-      <c r="S12" s="41" t="s">
+      <c r="R12" s="40"/>
+      <c r="S12" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="T12" s="42" t="s">
+      <c r="T12" s="36" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="51" x14ac:dyDescent="0.25">
-      <c r="A13" s="38"/>
-      <c r="B13" s="38"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
+      <c r="A13" s="37"/>
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="38"/>
       <c r="H13" s="23" t="s">
         <v>28</v>
       </c>
@@ -1118,14 +1118,14 @@
         <v>27</v>
       </c>
       <c r="L13" s="39"/>
-      <c r="M13" s="44"/>
+      <c r="M13" s="40"/>
       <c r="N13" s="39"/>
       <c r="O13" s="39"/>
       <c r="P13" s="39"/>
       <c r="Q13" s="39"/>
-      <c r="R13" s="44"/>
-      <c r="S13" s="41"/>
-      <c r="T13" s="42"/>
+      <c r="R13" s="40"/>
+      <c r="S13" s="35"/>
+      <c r="T13" s="36"/>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.7">
       <c r="A14" s="26"/>
@@ -1140,8 +1140,7 @@
       <c r="J14" s="29"/>
       <c r="K14" s="29"/>
       <c r="L14" s="29"/>
-      <c r="M14" s="30"/>
-      <c r="N14" s="29"/>
+      <c r="M14" s="17"/>
       <c r="O14" s="29"/>
       <c r="P14" s="29"/>
       <c r="Q14" s="29"/>
@@ -1422,6 +1421,18 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A10:T10"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A2:T2"/>
+    <mergeCell ref="A3:T3"/>
+    <mergeCell ref="A9:T9"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="D11:D13"/>
+    <mergeCell ref="H11:L11"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="L12:L13"/>
     <mergeCell ref="S11:T11"/>
     <mergeCell ref="S12:S13"/>
     <mergeCell ref="T12:T13"/>
@@ -1434,18 +1445,6 @@
     <mergeCell ref="N11:N13"/>
     <mergeCell ref="O11:O13"/>
     <mergeCell ref="M11:M13"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="D11:D13"/>
-    <mergeCell ref="H11:L11"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="L12:L13"/>
-    <mergeCell ref="A10:T10"/>
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="A2:T2"/>
-    <mergeCell ref="A3:T3"/>
-    <mergeCell ref="A9:T9"/>
   </mergeCells>
   <conditionalFormatting sqref="T4:T8 T11:T1048576">
     <cfRule type="cellIs" dxfId="3" priority="4" operator="lessThan">
@@ -1457,7 +1456,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N1:N1048576">
+  <conditionalFormatting sqref="N1:N13 N123:N1048576">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>